<commit_message>
Add media quizzes, bulk import, participant history, and hub UX polish.
Media questions and Excel/ZIP bulk import for admin/host, quiz history with downloads and clear, simplified lobby, and quiz layout updates for team chat and question stage.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/teams.xlsx
+++ b/data/teams.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,31 +425,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>emoji</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>color</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>created_by</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
@@ -461,7 +473,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>admin@citi.com</t>
+          <t>admin@abc.com</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -488,12 +500,201 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>admin@citi.com</t>
+          <t>admin@abc.com</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>2026-07-03 19:17:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Lone Wolf</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>🦁</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>#7c5cff</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>admin@abc.com</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-07-04 00:58:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Blue Sparks</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>#0088ce</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-07-04 09:47:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Red Arcs</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>🔥</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>#e21836</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-07-04 09:47:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Gold Rush</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>🏆</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>#ffc233</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-07-04 09:47:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Teal Titans</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>🌊</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>#00c9a7</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-07-04 09:47:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Ops Avengers</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>💜</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>#7c5cff</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-07-04 09:47:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CX Crusaders</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>🎯</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>#ff6b35</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-07-04 09:47:59</t>
         </is>
       </c>
     </row>

</xml_diff>